<commit_message>
fix(catalog): harden the pipeline for verticals it was not built for
- never ship a live formula: a scraped name beginning with = was stored by
  openpyxl as a formula and would evaluate on open. Both writers now force
  such cells back to text, preserving the characters exactly.
- merge-names no longer clobbers the English names translate-names wrote in
  place; re-running it alone reverted them and only showed up as a quiet drop
  in category matches.
- collapse whitespace at the export boundary, and flag rather than truncate a
  title long enough to suggest the scrape swallowed a paragraph.
- add an offline multi-vertical stress test covering food, electronics,
  apparel, non-Latin names, collisions and injection payloads.
- document stage ownership so new work lands at the right point in the pipeline.
</commit_message>
<xml_diff>
--- a/projects/splashstore/docs/splashstore-scan-curation-260816.xlsx
+++ b/projects/splashstore/docs/splashstore-scan-curation-260816.xlsx
@@ -2262,7 +2262,7 @@
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Calacatta 4-person Inflatable Spa</t>
+          <t>Calacatta 4-person inflatable spa</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Olive 8-person Inflatable Spa</t>
+          <t>Olive 8-person inflatable spa</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>SC750 Filter Replacement Filter Lamellar Filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
+          <t>SC750 Filter replacement filter lamellar filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Cristal Poolpflege CRISTAL Alkaline Edge Cleaner 1,0 l, (Gentle on Materials, for Liners, Plastic Surfaces</t>
+          <t>Cristal Poolpflege CRISTAL edge cleaner alkaline 1,0 l, (material-safe, for liners, plastic</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>AQUALITY Pool Cleaner for Greasy Residues 1L</t>
+          <t>AQUALITY Pool cleaner for greasy residue 1L</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Höfer Chemie GmbH Pool Care 1 L BAYZID® SPA Poolclear Turbidity Remover</t>
+          <t>Höfer Chemie GmbH pool care 1 L BAYZID® SPA Poolclear turbidity remover</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>HÖFER CHEMIE GMBH 1 l Hydrogen Peroxide 11,9%</t>
+          <t>HÖFER CHEMIE GMBH 1 l hydrogen peroxide 11,9%</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Astralpool Water Care Astralpool Chlorine Stabilizer 4,5 kg</t>
+          <t>Astralpool water care Astralpool Chlorine Stabilizer 4,5 kg</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Höfer Chemie GmbH 1 L Sauna Cleaner with Eucalyptus Scent - High-Concentrate Deep Cleaner</t>
+          <t>Höfer Chemie GmbH 1 L sauna cleaner with eucalyptus scent - high-concentrate heavy-duty cleaner</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>HTH Spa Spa Cleaner</t>
+          <t>HTH Spa spa cleaner</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>AIPER Scuba S3 Cordless Pool Robot, Automatic Floor and Wall Cleaning, WavePath™ Navigation, High-Performance Filtration and Smart Control</t>
+          <t>AIPER Scuba S3 cordless pool robot, automatic floor and wall cleaning, WavePath™ navigation, high-performance filtration and smart control</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>WAYS - Pool Maintenance - Scrub Brush - 15 x 9 x 8 cm - Handy scrub</t>
+          <t>WAYS - Pool maintenance - Scrub brush - 15 x 9 x 8 cm - Handy scrub</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>Headrest Pillow for INTEX Inflatable SPA 28506</t>
+          <t>Pillow for inflatable SPA INTEX 28506</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -4296,7 +4296,7 @@
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Active Oxygen Test Kit x1</t>
+          <t>Active oxygen test kit x1</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Darlly Filter Cartridge Pack of 2 Filter Cartridges Compatible with Intex Type H</t>
+          <t>Darlly filter cartridge pack of 2 filter cartridges compatible with Intex type H</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Spa Replacement Filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
+          <t>Spa replacement filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>1 x 1 kg BAYZID® 20g 5-in-1 Multitabs for Pools - HÖFER CHEMIE</t>
+          <t>1 x 1 kg BAYZID® multitabs 20g 5in1 for pools - HöFER CHEMIE</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Calacatta 4-person Inflatable Spa</t>
+          <t>Calacatta 4-person inflatable spa</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="AA9" s="18" t="inlineStr">
         <is>
-          <t>Calacatta 4-person Inflatable Spa</t>
+          <t>Calacatta 4-person inflatable spa</t>
         </is>
       </c>
       <c r="AB9" s="23" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Olive 8-person Inflatable Spa</t>
+          <t>Olive 8-person inflatable spa</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="AA12" s="18" t="inlineStr">
         <is>
-          <t>Olive 8-person Inflatable Spa</t>
+          <t>Olive 8-person inflatable spa</t>
         </is>
       </c>
       <c r="AB12" s="23" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>SC750 Filter Replacement Filter Lamellar Filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
+          <t>SC750 Filter replacement filter lamellar filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="AA13" s="18" t="inlineStr">
         <is>
-          <t>SC750 Filter Replacement Filter Lamellar Filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
+          <t>SC750 Filter replacement filter lamellar filter Arctic Fonteyn Rota Strong Spa - Darlly</t>
         </is>
       </c>
       <c r="AB13" s="23" t="inlineStr">
@@ -7076,12 +7076,12 @@
     <row r="17" ht="62" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>cristal-poolpflege-cristal-alkaline-edge-cleaner-1-0-l-gentle-on-materials-for-l</t>
+          <t>cristal-poolpflege-cristal-edge-cleaner-alkaline-1-0-l-material-safe-for-liners-</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Cristal Poolpflege CRISTAL Alkaline Edge Cleaner 1,0 l, (Gentle on Materials, for Liners, Plastic Surfaces</t>
+          <t>Cristal Poolpflege CRISTAL edge cleaner alkaline 1,0 l, (material-safe, for liners, plastic</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="AA17" s="18" t="inlineStr">
         <is>
-          <t>Cristal Poolpflege CRISTAL Alkaline Edge Cleaner 1,0 l, (Gentle on Materials, for Liners, Plastic Surfaces</t>
+          <t>Cristal Poolpflege CRISTAL edge cleaner alkaline 1,0 l, (material-safe, for liners, plastic</t>
         </is>
       </c>
       <c r="AB17" s="23" t="inlineStr">
@@ -7213,12 +7213,12 @@
     <row r="18" ht="76" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t>aquality-pool-cleaner-for-greasy-residues-1l</t>
+          <t>aquality-pool-cleaner-for-greasy-residue-1l</t>
         </is>
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>AQUALITY Pool Cleaner for Greasy Residues 1L</t>
+          <t>AQUALITY Pool cleaner for greasy residue 1L</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="AA18" s="18" t="inlineStr">
         <is>
-          <t>AQUALITY Pool Cleaner for Greasy Residues 1L</t>
+          <t>AQUALITY Pool cleaner for greasy residue 1L</t>
         </is>
       </c>
       <c r="AB18" s="23" t="inlineStr">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Höfer Chemie GmbH Pool Care 1 L BAYZID® SPA Poolclear Turbidity Remover</t>
+          <t>Höfer Chemie GmbH pool care 1 L BAYZID® SPA Poolclear turbidity remover</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="AA21" s="18" t="inlineStr">
         <is>
-          <t>Höfer Chemie GmbH Pool Care 1 L BAYZID® SPA Poolclear Turbidity Remover</t>
+          <t>Höfer Chemie GmbH pool care 1 L BAYZID® SPA Poolclear turbidity remover</t>
         </is>
       </c>
       <c r="AB21" s="23" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>HÖFER CHEMIE GMBH 1 l Hydrogen Peroxide 11,9%</t>
+          <t>HÖFER CHEMIE GMBH 1 l hydrogen peroxide 11,9%</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="AA22" s="18" t="inlineStr">
         <is>
-          <t>HÖFER CHEMIE GMBH 1 l Hydrogen Peroxide 11,9%</t>
+          <t>HÖFER CHEMIE GMBH 1 l hydrogen peroxide 11,9%</t>
         </is>
       </c>
       <c r="AB22" s="23" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Astralpool Water Care Astralpool Chlorine Stabilizer 4,5 kg</t>
+          <t>Astralpool water care Astralpool Chlorine Stabilizer 4,5 kg</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -8418,12 +8418,12 @@
     <row r="27" ht="62" customHeight="1">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>hofer-chemie-gmbh-1-l-sauna-cleaner-with-eucalyptus-scent-high-concentrate-deep-</t>
+          <t>hofer-chemie-gmbh-1-l-sauna-cleaner-with-eucalyptus-scent-high-concentrate-heavy</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Höfer Chemie GmbH 1 L Sauna Cleaner with Eucalyptus Scent - High-Concentrate Deep Cleaner</t>
+          <t>Höfer Chemie GmbH 1 L sauna cleaner with eucalyptus scent - high-concentrate heavy-duty cleaner</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>HTH Spa Spa Cleaner</t>
+          <t>HTH Spa spa cleaner</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -8657,7 +8657,7 @@
       </c>
       <c r="AA28" s="18" t="inlineStr">
         <is>
-          <t>HTH Spa Spa Cleaner</t>
+          <t>HTH Spa spa cleaner</t>
         </is>
       </c>
       <c r="AB28" s="23" t="inlineStr">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>AIPER Scuba S3 Cordless Pool Robot, Automatic Floor and Wall Cleaning, WavePath™ Navigation, High-Performance Filtration and Smart Control</t>
+          <t>AIPER Scuba S3 cordless pool robot, automatic floor and wall cleaning, WavePath™ navigation, high-performance filtration and smart control</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -8935,7 +8935,7 @@
       </c>
       <c r="AA30" s="18" t="inlineStr">
         <is>
-          <t>AIPER Scuba S3 Cordless Pool Robot, Automatic Floor and Wall Cleaning, WavePath™ Navigation, High-Performance Filtration…</t>
+          <t>AIPER Scuba S3 cordless pool robot, automatic floor and wall cleaning, WavePath™ navigation, high-performance filtration…</t>
         </is>
       </c>
       <c r="AB30" s="23" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>WAYS - Pool Maintenance - Scrub Brush - 15 x 9 x 8 cm - Handy scrub</t>
+          <t>WAYS - Pool maintenance - Scrub brush - 15 x 9 x 8 cm - Handy scrub</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
@@ -9792,12 +9792,12 @@
     <row r="37" ht="76" customHeight="1">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>headrest-pillow-for-intex-inflatable-spa-28506</t>
+          <t>pillow-for-inflatable-spa-intex-28506</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Headrest Pillow for INTEX Inflatable SPA 28506</t>
+          <t>Pillow for inflatable SPA INTEX 28506</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="AA37" s="18" t="inlineStr">
         <is>
-          <t>Headrest Pillow for INTEX Inflatable SPA 28506</t>
+          <t>Pillow for inflatable SPA INTEX 28506</t>
         </is>
       </c>
       <c r="AB37" s="23" t="inlineStr">
@@ -9950,7 +9950,7 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Active Oxygen Test Kit x1</t>
+          <t>Active oxygen test kit x1</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="AA38" s="18" t="inlineStr">
         <is>
-          <t>Active Oxygen Test Kit x1</t>
+          <t>Active oxygen test kit x1</t>
         </is>
       </c>
       <c r="AB38" s="23" t="inlineStr">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Darlly Filter Cartridge Pack of 2 Filter Cartridges Compatible with Intex Type H</t>
+          <t>Darlly filter cartridge pack of 2 filter cartridges compatible with Intex type H</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="AA39" s="18" t="inlineStr">
         <is>
-          <t>Darlly Filter Cartridge Pack of 2 Filter Cartridges Compatible with Intex Type H</t>
+          <t>Darlly filter cartridge pack of 2 filter cartridges compatible with Intex type H</t>
         </is>
       </c>
       <c r="AB39" s="23" t="inlineStr">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Spa Replacement Filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
+          <t>Spa replacement filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
@@ -10329,7 +10329,7 @@
       </c>
       <c r="AA40" s="18" t="inlineStr">
         <is>
-          <t>Spa Replacement Filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
+          <t>Spa replacement filter Ø 22 cm x 27 cm SC713, C-8465 - Darlly</t>
         </is>
       </c>
       <c r="AB40" s="23" t="inlineStr">
@@ -10360,12 +10360,12 @@
     <row r="41" ht="62" customHeight="1">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>1-x-1-kg-bayzid-20g-5-in-1-multitabs-for-pools-hofer-chemie</t>
+          <t>1-x-1-kg-bayzid-multitabs-20g-5in1-for-pools-hofer-chemie</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>1 x 1 kg BAYZID® 20g 5-in-1 Multitabs for Pools - HÖFER CHEMIE</t>
+          <t>1 x 1 kg BAYZID® multitabs 20g 5in1 for pools - HöFER CHEMIE</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
@@ -10478,7 +10478,7 @@
       </c>
       <c r="AA41" s="18" t="inlineStr">
         <is>
-          <t>1 x 1 kg BAYZID® 20g 5-in-1 Multitabs for Pools - HÖFER CHEMIE</t>
+          <t>1 x 1 kg BAYZID® multitabs 20g 5in1 for pools - HöFER CHEMIE</t>
         </is>
       </c>
       <c r="AB41" s="23" t="inlineStr">

</xml_diff>